<commit_message>
version 2025 01 08
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS C07/CAS C07.xlsx
+++ b/VALIDATION/CAS C07/CAS C07.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS C07\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB319E4-B09A-449E-AC81-15D577F9646D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE4B01E4-13B1-403A-92E8-8A9D851ED9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
   </bookViews>
   <sheets>
     <sheet name="Général" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <definedName name="AireA">Général!$E$15</definedName>
     <definedName name="Av">Général!$E$19</definedName>
     <definedName name="b">Général!$E$11</definedName>
+    <definedName name="b0">Général!$E$112</definedName>
     <definedName name="bb">Général!$E$47</definedName>
     <definedName name="beff">Général!$O$4</definedName>
     <definedName name="bei">Général!$O$7</definedName>
@@ -51,6 +52,7 @@
     <definedName name="Ht">Général!$E$10</definedName>
     <definedName name="hw">Général!$E$17</definedName>
     <definedName name="Iy">Général!$E$22</definedName>
+    <definedName name="ksfaa">Général!$E$113</definedName>
     <definedName name="Le">Général!$O$8</definedName>
     <definedName name="LL">Général!$E$4</definedName>
     <definedName name="mDalle">Général!$J$34</definedName>
@@ -123,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="159">
   <si>
     <t>Poutre</t>
   </si>
@@ -591,15 +593,25 @@
   </si>
   <si>
     <t>cm2/m</t>
+  </si>
+  <si>
+    <t>b0</t>
+  </si>
+  <si>
+    <t>ksf a-a</t>
+  </si>
+  <si>
+    <t>Critère</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -739,7 +751,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -809,6 +821,9 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
@@ -1155,7 +1170,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA8D444-109B-41E4-8631-33F090AACEB2}">
-  <dimension ref="C2:U123"/>
+  <dimension ref="C2:U125"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="3:21" x14ac:dyDescent="0.25">
@@ -2329,14 +2344,14 @@
         <v>123</v>
       </c>
       <c r="M87" s="13">
-        <v>148444</v>
+        <v>112303</v>
       </c>
       <c r="N87" s="13">
         <f>M87</f>
+        <v>112303</v>
+      </c>
+      <c r="O87" s="13">
         <v>148444</v>
-      </c>
-      <c r="O87" s="13">
-        <v>112303</v>
       </c>
     </row>
     <row r="88" spans="3:15" x14ac:dyDescent="0.25">
@@ -2368,15 +2383,15 @@
       </c>
       <c r="M89" s="20">
         <f>5/384*M88*LL^4/(Ey*M87/100)*1000^2</f>
-        <v>32.331403935900084</v>
+        <v>42.736195167188335</v>
       </c>
       <c r="N89" s="20">
         <f>5/384*N88*LL^4/(Ey*N87/100)*1000^2</f>
-        <v>8.023040488145174</v>
+        <v>10.604990269380359</v>
       </c>
       <c r="O89" s="20">
         <f>5/384*O88*LL^4/(Ey*O87/100)*1000^2</f>
-        <v>31.814970808141069</v>
+        <v>24.069121464435522</v>
       </c>
     </row>
     <row r="90" spans="3:15" x14ac:dyDescent="0.25">
@@ -2519,12 +2534,12 @@
       <c r="E106" s="12"/>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C107" s="31"/>
-      <c r="D107" s="32" t="s">
+      <c r="C107" s="32"/>
+      <c r="D107" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="E107" s="31"/>
-      <c r="F107" s="31"/>
+      <c r="E107" s="32"/>
+      <c r="F107" s="32"/>
     </row>
     <row r="108" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D108" s="2"/>
@@ -2555,7 +2570,7 @@
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D111" s="33" t="s">
+      <c r="D111" s="34" t="s">
         <v>25</v>
       </c>
       <c r="E111" s="14">
@@ -2563,112 +2578,146 @@
         <v>0.55200000000000005</v>
       </c>
     </row>
-    <row r="114" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D114" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E114" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F114" s="13" t="s">
-        <v>145</v>
+    <row r="112" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D112" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E112" s="14">
+        <f>2.5*dsc</f>
+        <v>55</v>
+      </c>
+      <c r="F112" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="113" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D113" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E113" s="31">
+        <f>(beff*1000-b0)/2/(beff*1000)</f>
+        <v>0.49214285714285716</v>
       </c>
     </row>
     <row r="115" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D115" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E115" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="F115" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="116" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D116" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="E115" s="13">
+      <c r="E116" s="13">
         <f>tc</f>
         <v>120</v>
       </c>
-      <c r="F115" s="13">
+      <c r="F116" s="13">
         <f>2*hsc+2.5*dsc+dsc</f>
         <v>277</v>
       </c>
     </row>
-    <row r="116" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D116" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E116" s="30">
-        <f>E110/E115</f>
-        <v>2.8974245444298874</v>
-      </c>
-      <c r="F116" s="30">
-        <f>E109/F115</f>
-        <v>2.5104039374121769</v>
-      </c>
-    </row>
     <row r="117" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D117" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E117" s="30">
-        <v>27</v>
+        <f>E109/E116*ksfaa</f>
+        <v>2.8518935873031319</v>
       </c>
       <c r="F117" s="30">
-        <v>27</v>
+        <f>E109/F116</f>
+        <v>2.5104039374121769</v>
       </c>
     </row>
     <row r="118" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D118" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E118" s="30">
-        <f>NuT*Fck/GammaC*SIN(E117*PI()/180)*COS(E117*PI()/180)</f>
-        <v>2.9771825392998066</v>
+        <v>27</v>
       </c>
       <c r="F118" s="30">
-        <f>NuT*Fck/GammaC*SIN(F117*PI()/180)*COS(F117*PI()/180)</f>
-        <v>2.9771825392998066</v>
+        <v>27</v>
       </c>
     </row>
     <row r="119" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D119" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E119" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="F119" s="13" t="s">
-        <v>150</v>
+        <v>148</v>
+      </c>
+      <c r="E119" s="30">
+        <f>NuT*Fck/GammaC*SIN(E118*PI()/180)*COS(E118*PI()/180)</f>
+        <v>2.9771825392998066</v>
+      </c>
+      <c r="F119" s="30">
+        <f>NuT*Fck/GammaC*SIN(F118*PI()/180)*COS(F118*PI()/180)</f>
+        <v>2.9771825392998066</v>
       </c>
     </row>
     <row r="120" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D120" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E120" s="30">
+        <f>E117/E119</f>
+        <v>0.95791693981043535</v>
+      </c>
+      <c r="F120" s="30">
+        <f>F117/F119</f>
+        <v>0.84321465152841801</v>
+      </c>
+    </row>
+    <row r="121" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D121" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E121" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="F121" s="13" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="122" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D122" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E120" s="20">
-        <f>E116*E115*TAN(E117*PI()/180)/100</f>
-        <v>1.7715738520521946</v>
-      </c>
-      <c r="F120" s="20">
-        <f>F116*F115*TAN(F117*PI()/180)/100</f>
-        <v>3.5431477041043902</v>
-      </c>
-    </row>
-    <row r="122" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D122" s="33" t="s">
+      <c r="E122" s="20">
+        <f>E117*E116*TAN(E118*PI()/180)/(Fsk/GammaS)*10</f>
+        <v>4.0105901190673041</v>
+      </c>
+      <c r="F122" s="20">
+        <f>F117*F116*TAN(F118*PI()/180)/(Fsk/GammaS)*10</f>
+        <v>8.1492397194400965</v>
+      </c>
+    </row>
+    <row r="124" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D124" s="34" t="s">
         <v>153</v>
       </c>
-      <c r="E122" s="20">
-        <f>F120/2</f>
-        <v>1.7715738520521951</v>
-      </c>
-      <c r="F122" t="s">
+      <c r="E124" s="20">
+        <f>F122/2</f>
+        <v>4.0746198597200483</v>
+      </c>
+      <c r="F124" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="123" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D123" s="33" t="s">
+    <row r="125" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D125" s="34" t="s">
         <v>154</v>
       </c>
-      <c r="E123" s="20">
-        <f>E120-E122</f>
-        <v>0</v>
-      </c>
-      <c r="F123" t="s">
+      <c r="E125" s="20">
+        <f>E122-E124</f>
+        <v>-6.4029740652744138E-2</v>
+      </c>
+      <c r="F125" t="s">
         <v>155</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Version 1.11 pour mise en service
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS C07/CAS C07.xlsx
+++ b/VALIDATION/CAS C07/CAS C07.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS C07\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV 23\VALIDATION\CAS C07\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE4B01E4-13B1-403A-92E8-8A9D851ED9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0CDFEA-71E3-4E9A-8503-3AA56DC57E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
   </bookViews>
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="168">
   <si>
     <t>Poutre</t>
   </si>
@@ -602,6 +602,33 @@
   </si>
   <si>
     <t>Critère</t>
+  </si>
+  <si>
+    <t>section dalle</t>
+  </si>
+  <si>
+    <t>Section nervure</t>
+  </si>
+  <si>
+    <t>Section nervure / UL</t>
+  </si>
+  <si>
+    <t>mm2/mm</t>
+  </si>
+  <si>
+    <t>volume dalle</t>
+  </si>
+  <si>
+    <t>m2</t>
+  </si>
+  <si>
+    <t>m3</t>
+  </si>
+  <si>
+    <t>volume dalle / UL</t>
+  </si>
+  <si>
+    <t>charge</t>
   </si>
 </sst>
 </file>
@@ -828,8 +855,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1443,7 +1470,7 @@
       </c>
       <c r="T14" s="23">
         <f>MEd/MplRd</f>
-        <v>0.94820659450469125</v>
+        <v>0.94429147867074081</v>
       </c>
     </row>
     <row r="15" spans="3:21" x14ac:dyDescent="0.25">
@@ -1472,7 +1499,7 @@
       </c>
       <c r="T15" s="23">
         <f>VEd/VplRd</f>
-        <v>0.27217483973946571</v>
+        <v>0.27105103820629506</v>
       </c>
     </row>
     <row r="16" spans="3:21" x14ac:dyDescent="0.25">
@@ -1826,8 +1853,8 @@
         <v>20</v>
       </c>
       <c r="J34" s="19">
-        <f>d*td*LL*RhoC/1000+d/ep*AVERAGE(bb,bt)*hp*RhoC/1000*LL</f>
-        <v>26320</v>
+        <f>d*td*LL*RhoC/1000+(d-b/1000)/ep*AVERAGE(bb,bt)*hp*RhoC/1000*LL</f>
+        <v>26073.599999999999</v>
       </c>
       <c r="K34" t="s">
         <v>87</v>
@@ -1976,6 +2003,10 @@
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
+      <c r="J43" s="19">
+        <f>d*td+d/ep*AVERAGE(bb,bt)*hp</f>
+        <v>783.33333333333337</v>
+      </c>
       <c r="O43" s="12"/>
     </row>
     <row r="44" spans="3:16" x14ac:dyDescent="0.25">
@@ -1991,7 +2022,16 @@
       <c r="F45" t="s">
         <v>6</v>
       </c>
-      <c r="O45" s="12"/>
+      <c r="M45" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N45" s="12">
+        <f>d*1000*tc</f>
+        <v>600000</v>
+      </c>
+      <c r="O45" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="46" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D46" s="2" t="s">
@@ -2003,7 +2043,23 @@
       <c r="F46" t="s">
         <v>6</v>
       </c>
-      <c r="O46" s="12"/>
+      <c r="J46">
+        <f>d*td*RhoC/1000+d/ep*AVERAGE(bb,bt)*hp*RhoC/1000</f>
+        <v>1880</v>
+      </c>
+      <c r="K46" t="s">
+        <v>135</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="N46" s="12">
+        <f>AVERAGE(bb,bt)*hp</f>
+        <v>27500</v>
+      </c>
+      <c r="O46" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="47" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D47" s="2" t="s">
@@ -2015,7 +2071,23 @@
       <c r="F47" t="s">
         <v>6</v>
       </c>
-      <c r="O47" s="12"/>
+      <c r="J47">
+        <f>d*td/1000+d/ep*AVERAGE(bb,bt)*hp*1000</f>
+        <v>183333.93333333335</v>
+      </c>
+      <c r="K47" t="s">
+        <v>12</v>
+      </c>
+      <c r="M47" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="N47" s="12">
+        <f>N46/hp*1000</f>
+        <v>125000</v>
+      </c>
+      <c r="O47" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="48" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D48" s="2" t="s">
@@ -2027,7 +2099,23 @@
       <c r="F48" t="s">
         <v>6</v>
       </c>
-      <c r="O48" s="12"/>
+      <c r="J48">
+        <f>J47/100</f>
+        <v>1833.3393333333336</v>
+      </c>
+      <c r="K48" t="s">
+        <v>13</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="N48" s="34">
+        <f>N45*LL/1000^2+N46/1000^2*LL/(ep/1000)*d</f>
+        <v>10.966666666666667</v>
+      </c>
+      <c r="O48" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="49" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D49" s="2" t="s">
@@ -2039,7 +2127,16 @@
       <c r="F49" t="s">
         <v>6</v>
       </c>
-      <c r="O49" s="12"/>
+      <c r="M49" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="N49" s="34">
+        <f>N48/LL</f>
+        <v>0.78333333333333333</v>
+      </c>
+      <c r="O49" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="50" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D50" s="2" t="s">
@@ -2051,7 +2148,16 @@
       <c r="F50" t="s">
         <v>132</v>
       </c>
-      <c r="O50" s="12"/>
+      <c r="M50" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="N50" s="12">
+        <f>N49*RhoC*g/1000</f>
+        <v>18.442799999999998</v>
+      </c>
+      <c r="O50" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="51" spans="3:15" x14ac:dyDescent="0.25">
       <c r="O51" s="12"/>
@@ -2091,7 +2197,7 @@
       </c>
       <c r="E59" s="16">
         <f>mDalle/LL*g/1000</f>
-        <v>18.442799999999998</v>
+        <v>18.270144000000002</v>
       </c>
       <c r="F59" t="s">
         <v>88</v>
@@ -2108,7 +2214,7 @@
       </c>
       <c r="N59" s="17">
         <f>GammaG*(q_G1+q_G2)+GammaQ*q_Q1</f>
-        <v>56.451280722662688</v>
+        <v>56.218195122662692</v>
       </c>
       <c r="O59" t="s">
         <v>88</v>
@@ -2151,7 +2257,7 @@
       </c>
       <c r="E62" s="16">
         <f>q1Dalle+q1Pro+q1Bac</f>
-        <v>20.149096831601987</v>
+        <v>19.976440831601991</v>
       </c>
       <c r="F62" t="s">
         <v>88</v>
@@ -2161,7 +2267,7 @@
       </c>
       <c r="N62" s="18">
         <f>qULS*LL^2/8</f>
-        <v>1383.0563777052359</v>
+        <v>1377.345780505236</v>
       </c>
       <c r="O62" t="s">
         <v>69</v>
@@ -2195,7 +2301,7 @@
       </c>
       <c r="N63" s="18">
         <f>qULS*LL/2</f>
-        <v>395.15896505863884</v>
+        <v>393.52736585863886</v>
       </c>
       <c r="O63" t="s">
         <v>54</v>
@@ -2242,15 +2348,15 @@
       </c>
       <c r="E72" s="20">
         <f>q_G1</f>
-        <v>20.149096831601987</v>
+        <v>19.976440831601991</v>
       </c>
       <c r="F72" s="20">
         <f>E72*LL^2/8</f>
-        <v>493.65287237424872</v>
+        <v>489.42280037424877</v>
       </c>
       <c r="G72" s="20">
         <f>E72*LL/2</f>
-        <v>141.04367782121392</v>
+        <v>139.83508582121394</v>
       </c>
     </row>
     <row r="73" spans="4:7" x14ac:dyDescent="0.25">
@@ -2293,15 +2399,15 @@
       </c>
       <c r="E75" s="20">
         <f>GammaG*(E72+E73)+GammaQ*E74</f>
-        <v>56.451280722662688</v>
+        <v>56.218195122662692</v>
       </c>
       <c r="F75" s="20">
         <f>GammaG*(F72+F73)+GammaQ*F74</f>
-        <v>1383.0563777052359</v>
+        <v>1377.3457805052358</v>
       </c>
       <c r="G75" s="20">
         <f>GammaG*(G72+G73)+GammaQ*G74</f>
-        <v>395.15896505863884</v>
+        <v>393.52736585863886</v>
       </c>
     </row>
     <row r="84" spans="3:15" x14ac:dyDescent="0.25">
@@ -2366,7 +2472,7 @@
       </c>
       <c r="M88" s="20">
         <f>E72</f>
-        <v>20.149096831601987</v>
+        <v>19.976440831601991</v>
       </c>
       <c r="N88" s="20">
         <f>E73</f>
@@ -2383,7 +2489,7 @@
       </c>
       <c r="M89" s="20">
         <f>5/384*M88*LL^4/(Ey*M87/100)*1000^2</f>
-        <v>42.736195167188335</v>
+        <v>42.369992127198309</v>
       </c>
       <c r="N89" s="20">
         <f>5/384*N88*LL^4/(Ey*N87/100)*1000^2</f>
@@ -2570,7 +2676,7 @@
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D111" s="34" t="s">
+      <c r="D111" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E111" s="14">
@@ -2698,7 +2804,7 @@
       </c>
     </row>
     <row r="124" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D124" s="34" t="s">
+      <c r="D124" s="2" t="s">
         <v>153</v>
       </c>
       <c r="E124" s="20">
@@ -2710,7 +2816,7 @@
       </c>
     </row>
     <row r="125" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D125" s="34" t="s">
+      <c r="D125" s="2" t="s">
         <v>154</v>
       </c>
       <c r="E125" s="20">

</xml_diff>